<commit_message>
Silver layer jobs created, terraform testenv created and some modifications in file structure
</commit_message>
<xml_diff>
--- a/Documentation/data_dictionary.xlsx
+++ b/Documentation/data_dictionary.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="18229"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Prakhar\Downloads\Logistic\Case Study\HR Analytics Case Study\PA-I_Case_Study_HR_Analytics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MarcoPortilho\Documents\Projects\HR_Analytics_ETL\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F660BA60-364A-42E2-9CF5-98F0C0F3776F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7530"/>
+    <workbookView xWindow="5775" yWindow="375" windowWidth="11685" windowHeight="13762" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data_dictionary" sheetId="1" r:id="rId1"/>
@@ -258,7 +259,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -866,9 +867,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -906,7 +907,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1012,7 +1013,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1154,23 +1155,23 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C53"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="23.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="72.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.73046875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="72.265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.1328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1181,7 +1182,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -1190,7 +1191,7 @@
       </c>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
@@ -1199,7 +1200,7 @@
       </c>
       <c r="C3" s="2"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -1208,7 +1209,7 @@
       </c>
       <c r="C4" s="2"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
@@ -1217,7 +1218,7 @@
       </c>
       <c r="C5" s="2"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
@@ -1226,7 +1227,7 @@
       </c>
       <c r="C6" s="2"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
         <v>13</v>
       </c>
@@ -1237,35 +1238,35 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A8" s="4"/>
       <c r="B8" s="4"/>
       <c r="C8" s="2" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A9" s="4"/>
       <c r="B9" s="4"/>
       <c r="C9" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A10" s="4"/>
       <c r="B10" s="4"/>
       <c r="C10" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A11" s="5"/>
       <c r="B11" s="5"/>
       <c r="C11" s="2" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A12" s="2" t="s">
         <v>20</v>
       </c>
@@ -1274,7 +1275,7 @@
       </c>
       <c r="C12" s="2"/>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A13" s="2" t="s">
         <v>22</v>
       </c>
@@ -1283,7 +1284,7 @@
       </c>
       <c r="C13" s="2"/>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A14" s="2" t="s">
         <v>24</v>
       </c>
@@ -1292,7 +1293,7 @@
       </c>
       <c r="C14" s="2"/>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A15" s="3" t="s">
         <v>26</v>
       </c>
@@ -1303,28 +1304,28 @@
         <v>28</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A16" s="4"/>
       <c r="B16" s="4"/>
       <c r="C16" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A17" s="4"/>
       <c r="B17" s="4"/>
       <c r="C17" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A18" s="5"/>
       <c r="B18" s="5"/>
       <c r="C18" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A19" s="2" t="s">
         <v>32</v>
       </c>
@@ -1333,7 +1334,7 @@
       </c>
       <c r="C19" s="2"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A20" s="3" t="s">
         <v>34</v>
       </c>
@@ -1344,28 +1345,28 @@
         <v>28</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A21" s="4"/>
       <c r="B21" s="4"/>
       <c r="C21" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A22" s="4"/>
       <c r="B22" s="4"/>
       <c r="C22" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A23" s="5"/>
       <c r="B23" s="5"/>
       <c r="C23" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A24" s="2" t="s">
         <v>36</v>
       </c>
@@ -1374,7 +1375,7 @@
       </c>
       <c r="C24" s="2"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A25" s="2" t="s">
         <v>38</v>
       </c>
@@ -1383,7 +1384,7 @@
       </c>
       <c r="C25" s="2"/>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A26" s="3" t="s">
         <v>40</v>
       </c>
@@ -1394,28 +1395,28 @@
         <v>28</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A27" s="4"/>
       <c r="B27" s="4"/>
       <c r="C27" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A28" s="4"/>
       <c r="B28" s="4"/>
       <c r="C28" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A29" s="5"/>
       <c r="B29" s="5"/>
       <c r="C29" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A30" s="2" t="s">
         <v>42</v>
       </c>
@@ -1424,7 +1425,7 @@
       </c>
       <c r="C30" s="2"/>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A31" s="2" t="s">
         <v>44</v>
       </c>
@@ -1433,7 +1434,7 @@
       </c>
       <c r="C31" s="2"/>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A32" s="2" t="s">
         <v>46</v>
       </c>
@@ -1442,7 +1443,7 @@
       </c>
       <c r="C32" s="2"/>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A33" s="2" t="s">
         <v>48</v>
       </c>
@@ -1451,7 +1452,7 @@
       </c>
       <c r="C33" s="2"/>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A34" s="2" t="s">
         <v>50</v>
       </c>
@@ -1460,7 +1461,7 @@
       </c>
       <c r="C34" s="2"/>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A35" s="3" t="s">
         <v>52</v>
       </c>
@@ -1471,28 +1472,28 @@
         <v>28</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A36" s="4"/>
       <c r="B36" s="4"/>
       <c r="C36" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A37" s="4"/>
       <c r="B37" s="4"/>
       <c r="C37" s="2" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A38" s="5"/>
       <c r="B38" s="5"/>
       <c r="C38" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A39" s="3" t="s">
         <v>57</v>
       </c>
@@ -1503,28 +1504,28 @@
         <v>28</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A40" s="4"/>
       <c r="B40" s="4"/>
       <c r="C40" s="2" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A41" s="4"/>
       <c r="B41" s="4"/>
       <c r="C41" s="2" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A42" s="5"/>
       <c r="B42" s="5"/>
       <c r="C42" s="2" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A43" s="2" t="s">
         <v>59</v>
       </c>
@@ -1533,7 +1534,7 @@
       </c>
       <c r="C43" s="2"/>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A44" s="2" t="s">
         <v>61</v>
       </c>
@@ -1542,7 +1543,7 @@
       </c>
       <c r="C44" s="2"/>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A45" s="2" t="s">
         <v>63</v>
       </c>
@@ -1551,7 +1552,7 @@
       </c>
       <c r="C45" s="2"/>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A46" s="2" t="s">
         <v>65</v>
       </c>
@@ -1560,7 +1561,7 @@
       </c>
       <c r="C46" s="2"/>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A47" s="3" t="s">
         <v>67</v>
       </c>
@@ -1571,28 +1572,28 @@
         <v>69</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A48" s="4"/>
       <c r="B48" s="4"/>
       <c r="C48" s="2" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A49" s="4"/>
       <c r="B49" s="4"/>
       <c r="C49" s="2" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A50" s="5"/>
       <c r="B50" s="5"/>
       <c r="C50" s="2" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A51" s="2" t="s">
         <v>72</v>
       </c>
@@ -1601,7 +1602,7 @@
       </c>
       <c r="C51" s="2"/>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A52" s="2" t="s">
         <v>74</v>
       </c>
@@ -1610,7 +1611,7 @@
       </c>
       <c r="C52" s="2"/>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A53" s="2" t="s">
         <v>76</v>
       </c>
@@ -1621,11 +1622,6 @@
     </row>
   </sheetData>
   <mergeCells count="14">
-    <mergeCell ref="A39:A42"/>
-    <mergeCell ref="B39:B42"/>
-    <mergeCell ref="B47:B50"/>
-    <mergeCell ref="A47:A50"/>
-    <mergeCell ref="B26:B29"/>
     <mergeCell ref="B20:B23"/>
     <mergeCell ref="A20:A23"/>
     <mergeCell ref="A26:A29"/>
@@ -1633,6 +1629,11 @@
     <mergeCell ref="B7:B11"/>
     <mergeCell ref="A15:A18"/>
     <mergeCell ref="B15:B18"/>
+    <mergeCell ref="A39:A42"/>
+    <mergeCell ref="B39:B42"/>
+    <mergeCell ref="B47:B50"/>
+    <mergeCell ref="A47:A50"/>
+    <mergeCell ref="B26:B29"/>
     <mergeCell ref="B35:B38"/>
     <mergeCell ref="A35:A38"/>
   </mergeCells>

</xml_diff>